<commit_message>
chore(weekly-sync): auto-pull through 2026-07-27
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week30.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week30.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="SD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SB" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +36,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +44,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,42 +419,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
@@ -969,10 +958,10 @@
         <v>69025</v>
       </c>
       <c r="G19" t="n">
-        <v>41540.69</v>
+        <v>48453.41</v>
       </c>
       <c r="H19" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20">
@@ -1053,10 +1042,10 @@
         <v>5700</v>
       </c>
       <c r="G22" t="n">
-        <v>8638.98</v>
+        <v>7199.15</v>
       </c>
       <c r="H22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23">
@@ -1252,7 +1241,7 @@
         <v>37569.47</v>
       </c>
       <c r="H29" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="30">
@@ -1613,10 +1602,10 @@
         <v>11356</v>
       </c>
       <c r="G42" t="n">
-        <v>41041.5</v>
+        <v>45479.64</v>
       </c>
       <c r="H42" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43">
@@ -1806,7 +1795,7 @@
         <v>540</v>
       </c>
       <c r="F49" t="n">
-        <v>83085</v>
+        <v>83086</v>
       </c>
       <c r="G49" t="n">
         <v>3107.63</v>
@@ -2170,7 +2159,7 @@
         <v>146</v>
       </c>
       <c r="F62" t="n">
-        <v>11515</v>
+        <v>11514</v>
       </c>
       <c r="G62" t="n">
         <v>6355.08</v>
@@ -2198,7 +2187,7 @@
         <v>621</v>
       </c>
       <c r="F63" t="n">
-        <v>46634</v>
+        <v>46633</v>
       </c>
       <c r="G63" t="n">
         <v>24571.18</v>
@@ -2226,7 +2215,7 @@
         <v>218</v>
       </c>
       <c r="F64" t="n">
-        <v>21730</v>
+        <v>21729</v>
       </c>
       <c r="G64" t="n">
         <v>4660.17</v>
@@ -2537,10 +2526,10 @@
         <v>37428</v>
       </c>
       <c r="G75" t="n">
-        <v>14116.96</v>
+        <v>17082.21</v>
       </c>
       <c r="H75" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="76">
@@ -2730,7 +2719,7 @@
         <v>131</v>
       </c>
       <c r="F82" t="n">
-        <v>36917</v>
+        <v>36915</v>
       </c>
       <c r="G82" t="n">
         <v>7662.69</v>
@@ -2898,7 +2887,7 @@
         <v>2077</v>
       </c>
       <c r="F88" t="n">
-        <v>277181</v>
+        <v>277171</v>
       </c>
       <c r="G88" t="n">
         <v>7641.52</v>
@@ -2954,7 +2943,7 @@
         <v>38</v>
       </c>
       <c r="F90" t="n">
-        <v>20327</v>
+        <v>20326</v>
       </c>
       <c r="G90" t="n">
         <v>0</v>
@@ -3094,7 +3083,7 @@
         <v>652</v>
       </c>
       <c r="F95" t="n">
-        <v>134346</v>
+        <v>134345</v>
       </c>
       <c r="G95" t="n">
         <v>13639.83</v>
@@ -3290,7 +3279,7 @@
         <v>721</v>
       </c>
       <c r="F102" t="n">
-        <v>82072</v>
+        <v>82071</v>
       </c>
       <c r="G102" t="n">
         <v>11620.31</v>
@@ -3598,7 +3587,7 @@
         <v>33</v>
       </c>
       <c r="F113" t="n">
-        <v>5637</v>
+        <v>5636</v>
       </c>
       <c r="G113" t="n">
         <v>0</v>
@@ -3738,7 +3727,7 @@
         <v>93</v>
       </c>
       <c r="F118" t="n">
-        <v>15790</v>
+        <v>15782</v>
       </c>
       <c r="G118" t="n">
         <v>2668.64</v>
@@ -3769,10 +3758,10 @@
         <v>6752</v>
       </c>
       <c r="G119" t="n">
-        <v>5520.33</v>
+        <v>8188.969999999999</v>
       </c>
       <c r="H119" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="120">
@@ -3822,7 +3811,7 @@
         <v>162</v>
       </c>
       <c r="F121" t="n">
-        <v>40192</v>
+        <v>40184</v>
       </c>
       <c r="G121" t="n">
         <v>0</v>
@@ -3853,7 +3842,7 @@
         <v>17309</v>
       </c>
       <c r="G122" t="n">
-        <v>21746.58</v>
+        <v>20391.5</v>
       </c>
       <c r="H122" t="n">
         <v>9</v>
@@ -3962,7 +3951,7 @@
         <v>81</v>
       </c>
       <c r="F126" t="n">
-        <v>19451</v>
+        <v>19450</v>
       </c>
       <c r="G126" t="n">
         <v>5507.63</v>
@@ -3990,7 +3979,7 @@
         <v>97</v>
       </c>
       <c r="F127" t="n">
-        <v>14590</v>
+        <v>14582</v>
       </c>
       <c r="G127" t="n">
         <v>0</v>
@@ -4158,7 +4147,7 @@
         <v>447</v>
       </c>
       <c r="F133" t="n">
-        <v>54025</v>
+        <v>54016</v>
       </c>
       <c r="G133" t="n">
         <v>10777.97</v>
@@ -4320,19 +4309,19 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>2489.73</v>
+        <v>2486.99</v>
       </c>
       <c r="E139" t="n">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="F139" t="n">
-        <v>95894</v>
+        <v>95893</v>
       </c>
       <c r="G139" t="n">
-        <v>25844.07</v>
+        <v>32974.59</v>
       </c>
       <c r="H139" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="140">
@@ -4354,13 +4343,13 @@
         <v>818</v>
       </c>
       <c r="F140" t="n">
-        <v>109397</v>
+        <v>109395</v>
       </c>
       <c r="G140" t="n">
-        <v>0</v>
+        <v>1355.08</v>
       </c>
       <c r="H140" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="141">
@@ -4410,13 +4399,13 @@
         <v>560</v>
       </c>
       <c r="F142" t="n">
-        <v>59060</v>
+        <v>59059</v>
       </c>
       <c r="G142" t="n">
-        <v>9149.99</v>
+        <v>12115.24</v>
       </c>
       <c r="H142" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="143">
@@ -4914,7 +4903,7 @@
         <v>347</v>
       </c>
       <c r="F160" t="n">
-        <v>57111</v>
+        <v>57110</v>
       </c>
       <c r="G160" t="n">
         <v>23209.28</v>
@@ -5586,7 +5575,7 @@
         <v>89</v>
       </c>
       <c r="F184" t="n">
-        <v>14586</v>
+        <v>14585</v>
       </c>
       <c r="G184" t="n">
         <v>0</v>
@@ -5925,10 +5914,10 @@
         <v>55188</v>
       </c>
       <c r="G196" t="n">
-        <v>16947.46</v>
+        <v>25421.19</v>
       </c>
       <c r="H196" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="197">
@@ -5978,7 +5967,7 @@
         <v>181</v>
       </c>
       <c r="F198" t="n">
-        <v>35455</v>
+        <v>35453</v>
       </c>
       <c r="G198" t="n">
         <v>0</v>
@@ -6118,7 +6107,7 @@
         <v>272</v>
       </c>
       <c r="F203" t="n">
-        <v>33035</v>
+        <v>33034</v>
       </c>
       <c r="G203" t="n">
         <v>5083.9</v>
@@ -6174,13 +6163,13 @@
         <v>443</v>
       </c>
       <c r="F205" t="n">
-        <v>29987</v>
+        <v>29986</v>
       </c>
       <c r="G205" t="n">
-        <v>17344.91</v>
+        <v>19734.74</v>
       </c>
       <c r="H205" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="206">
@@ -6202,7 +6191,7 @@
         <v>181</v>
       </c>
       <c r="F206" t="n">
-        <v>19970</v>
+        <v>19969</v>
       </c>
       <c r="G206" t="n">
         <v>7130.52</v>
@@ -6286,7 +6275,7 @@
         <v>87</v>
       </c>
       <c r="F209" t="n">
-        <v>67307</v>
+        <v>67306</v>
       </c>
       <c r="G209" t="n">
         <v>4235.6</v>
@@ -6538,7 +6527,7 @@
         <v>82</v>
       </c>
       <c r="F218" t="n">
-        <v>8132</v>
+        <v>8131</v>
       </c>
       <c r="G218" t="n">
         <v>0</v>
@@ -6874,7 +6863,7 @@
         <v>176</v>
       </c>
       <c r="F230" t="n">
-        <v>17197</v>
+        <v>17196</v>
       </c>
       <c r="G230" t="n">
         <v>5080.5</v>
@@ -6930,7 +6919,7 @@
         <v>71</v>
       </c>
       <c r="F232" t="n">
-        <v>48963</v>
+        <v>48960</v>
       </c>
       <c r="G232" t="n">
         <v>1609.32</v>
@@ -7070,7 +7059,7 @@
         <v>461</v>
       </c>
       <c r="F237" t="n">
-        <v>68943</v>
+        <v>68941</v>
       </c>
       <c r="G237" t="n">
         <v>27358.44</v>
@@ -7098,7 +7087,7 @@
         <v>39</v>
       </c>
       <c r="F238" t="n">
-        <v>9996</v>
+        <v>9992</v>
       </c>
       <c r="G238" t="n">
         <v>0</v>
@@ -7322,7 +7311,7 @@
         <v>593</v>
       </c>
       <c r="F246" t="n">
-        <v>119252</v>
+        <v>119244</v>
       </c>
       <c r="G246" t="n">
         <v>6249.15</v>
@@ -7941,10 +7930,10 @@
         <v>39389</v>
       </c>
       <c r="G268" t="n">
-        <v>12623.73</v>
+        <v>15013.56</v>
       </c>
       <c r="H268" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="269">
@@ -9562,7 +9551,7 @@
         <v>197</v>
       </c>
       <c r="F326" t="n">
-        <v>45441</v>
+        <v>45439</v>
       </c>
       <c r="G326" t="n">
         <v>4743.22</v>
@@ -9674,7 +9663,7 @@
         <v>104</v>
       </c>
       <c r="F330" t="n">
-        <v>16750</v>
+        <v>16749</v>
       </c>
       <c r="G330" t="n">
         <v>9063.559999999999</v>
@@ -10034,42 +10023,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
@@ -10424,19 +10413,19 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>9189.969999999999</v>
+        <v>9187.77</v>
       </c>
       <c r="E14" t="n">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="F14" t="n">
-        <v>316539</v>
+        <v>316538</v>
       </c>
       <c r="G14" t="n">
-        <v>38710.99</v>
+        <v>42777.09</v>
       </c>
       <c r="H14" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
@@ -10816,19 +10805,19 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2251.14</v>
+        <v>2250.53</v>
       </c>
       <c r="E28" t="n">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="F28" t="n">
         <v>173139</v>
       </c>
       <c r="G28" t="n">
-        <v>29170.34</v>
+        <v>36796.61</v>
       </c>
       <c r="H28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
@@ -11077,10 +11066,10 @@
         <v>40649</v>
       </c>
       <c r="G37" t="n">
-        <v>13557.63</v>
+        <v>15947.46</v>
       </c>
       <c r="H37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38">
@@ -11152,13 +11141,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>4969.2</v>
+        <v>4963.79</v>
       </c>
       <c r="E40" t="n">
-        <v>4044</v>
+        <v>4038</v>
       </c>
       <c r="F40" t="n">
-        <v>980006</v>
+        <v>979957</v>
       </c>
       <c r="G40" t="n">
         <v>61792.36</v>
@@ -11305,6 +11294,661 @@
       </c>
       <c r="H45" t="n">
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Portfolio name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Campaign Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Advertised ASIN</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Clicks</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>14 Day Total Sales (₹)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>14 Day Total Units (#)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Audio Array-B0BLJVJ2GN-AA 05 Suspension-SB-PT</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>B0BLJVJ2GN</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>10399</v>
+      </c>
+      <c r="E2" t="n">
+        <v>139</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1804.086933445784</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2309.798461560832</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Audio Array-B0BLJVJ2GN-AA 05 Suspension-SB-PT</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>B0BQ7H7418</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6938</v>
+      </c>
+      <c r="E3" t="n">
+        <v>92</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1203.643066554216</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1541.041538439168</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Audio Array-B0BPLZ5CGV-AI 04 Audio Interface-SBV -PT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>B0BPLZ5CGV</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>72989</v>
+      </c>
+      <c r="E4" t="n">
+        <v>638</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4465.89</v>
+      </c>
+      <c r="G4" t="n">
+        <v>8132.2</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Audio Array-B0CKHVHVQ1-AM W45 Wireless-SBV-KT-Phrase</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>B0CKHVHVQ1</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>51228</v>
+      </c>
+      <c r="E5" t="n">
+        <v>183</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2793.31</v>
+      </c>
+      <c r="G5" t="n">
+        <v>18227.12</v>
+      </c>
+      <c r="H5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Audio Array-B0CKHVHVQ1-AM W45 Wireless-SBV-PT</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>B0CKHVHVQ1</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>46121</v>
+      </c>
+      <c r="E6" t="n">
+        <v>260</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1276.910743233532</v>
+      </c>
+      <c r="G6" t="n">
+        <v>9013.560000000001</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Audio Array-B0CKHVHVQ1-AM W45 Wireless-SBV-PT</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>B0H3LHF2WW</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>10837</v>
+      </c>
+      <c r="E7" t="n">
+        <v>61</v>
+      </c>
+      <c r="F7" t="n">
+        <v>300.0192567664689</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2117.8</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>B0B4DPX2J2</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5279</v>
+      </c>
+      <c r="E8" t="n">
+        <v>62</v>
+      </c>
+      <c r="F8" t="n">
+        <v>989.4322359269896</v>
+      </c>
+      <c r="G8" t="n">
+        <v>7514.641577656712</v>
+      </c>
+      <c r="H8" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>B0B4K87PR4</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>14089</v>
+      </c>
+      <c r="E9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F9" t="n">
+        <v>475.0580237967505</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3678.058248518646</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>B0BPLWW72Y</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>6362</v>
+      </c>
+      <c r="E10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F10" t="n">
+        <v>214.5295907135917</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1660.959906264091</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>B0BPLZ5CGV</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>6766</v>
+      </c>
+      <c r="E11" t="n">
+        <v>74</v>
+      </c>
+      <c r="F11" t="n">
+        <v>704.055136395746</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4066.1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>B0BQ7H7418</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1832</v>
+      </c>
+      <c r="E12" t="n">
+        <v>20</v>
+      </c>
+      <c r="F12" t="n">
+        <v>190.6148636042539</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1100.85</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>B0CBCB82MT</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1552</v>
+      </c>
+      <c r="E13" t="n">
+        <v>18</v>
+      </c>
+      <c r="F13" t="n">
+        <v>290.9332001570898</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2209.609352552481</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>B0CH4RT4P8</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>3202</v>
+      </c>
+      <c r="E14" t="n">
+        <v>38</v>
+      </c>
+      <c r="F14" t="n">
+        <v>600.2445639159205</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4558.799069790806</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>B0CKHVHVQ1</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>101821</v>
+      </c>
+      <c r="E15" t="n">
+        <v>436</v>
+      </c>
+      <c r="F15" t="n">
+        <v>3433.242385489658</v>
+      </c>
+      <c r="G15" t="n">
+        <v>26581.31184521726</v>
+      </c>
+      <c r="H15" t="n">
+        <v>7</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Audio Array_B0DXFPM4N2_Studio Monitor_SB Video</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>B0DXFPM4N2</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>169219</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1056</v>
+      </c>
+      <c r="F16" t="n">
+        <v>6532.27</v>
+      </c>
+      <c r="G16" t="n">
+        <v>7671.19</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Audio Array_B0GKPXQ8G3_Wireless Mic_SBV</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>B0GKPXQ8G3</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>245</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Audio Array_Studio Headphones_SB_KT_Phrase</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>B0FG88HVQ8</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>22859</v>
+      </c>
+      <c r="E18" t="n">
+        <v>59</v>
+      </c>
+      <c r="F18" t="n">
+        <v>658.1576960122716</v>
+      </c>
+      <c r="G18" t="n">
+        <v>3388.14</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Audio Array_Studio Headphones_SB_KT_Phrase</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>B0FQBXS6Y2</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>17781</v>
+      </c>
+      <c r="E19" t="n">
+        <v>46</v>
+      </c>
+      <c r="F19" t="n">
+        <v>511.9723039877287</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2635.59</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>